<commit_message>
add resident bulk import + migrate to bun
</commit_message>
<xml_diff>
--- a/frontend/public/excel/room_import_template.xlsx
+++ b/frontend/public/excel/room_import_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Docs\sdx\room-management-system\frontend\public\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6CF680E3-8C10-4E4C-9FA9-3303CBB5189A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005B433B-5252-4B11-8B02-21D350C693F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{4E3B61D4-F00A-4715-A597-5B07298220D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E3B61D4-F00A-4715-A597-5B07298220D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>siteName</t>
   </si>
@@ -63,6 +63,18 @@
   </si>
   <si>
     <t>numberOfBeds</t>
+  </si>
+  <si>
+    <t>DSLNG</t>
+  </si>
+  <si>
+    <t>EAST CAMP</t>
+  </si>
+  <si>
+    <t>ROOM</t>
+  </si>
+  <si>
+    <t>A</t>
   </si>
 </sst>
 </file>
@@ -434,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62302EA5-A0CE-41E1-B63E-BDCBB0E50603}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.109375" customWidth="1"/>
@@ -471,6 +483,32 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>101</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>